<commit_message>
feat: add cccd, msdvqhns, and sohochieu fields on invoice_bh
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/einvoices1/MauUploadHDBH-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/einvoices1/MauUploadHDBH-TT78.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="23040" windowHeight="8940"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
     <author>ASIA</author>
   </authors>
   <commentList>
-    <comment ref="J1" authorId="0">
+    <comment ref="M1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -51,7 +51,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0">
+    <comment ref="T1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -73,7 +73,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0">
+    <comment ref="U1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -103,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="56">
   <si>
     <t>MaHD(*)</t>
   </si>
@@ -117,6 +117,9 @@
     <t>TenDonVi</t>
   </si>
   <si>
+    <t>MaSoĐVQHNS</t>
+  </si>
+  <si>
     <t>DiaChiKhachHang</t>
   </si>
   <si>
@@ -124,6 +127,12 @@
   </si>
   <si>
     <t>SoDienThoaiKH</t>
+  </si>
+  <si>
+    <t>SoCCCD</t>
+  </si>
+  <si>
+    <t>SoHoChieu</t>
   </si>
   <si>
     <t>SoTaiKhoan</t>
@@ -274,7 +283,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,13 +293,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -459,7 +461,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -546,19 +548,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -780,97 +770,103 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -879,10 +875,10 @@
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -891,10 +887,10 @@
     <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -903,10 +899,10 @@
     <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -915,19 +911,14 @@
     <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1264,29 +1255,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11.8190476190476" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="12.7238095238095" customWidth="1"/>
-    <col min="5" max="6" width="19.1809523809524" customWidth="1"/>
-    <col min="7" max="7" width="15.2666666666667" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="12.8190476190476" customWidth="1"/>
-    <col min="10" max="10" width="22.1809523809524" style="2" customWidth="1"/>
-    <col min="11" max="11" width="11.5428571428571" customWidth="1"/>
-    <col min="12" max="12" width="15.4571428571429" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="13.8190476190476" customWidth="1"/>
-    <col min="15" max="15" width="9.18095238095238" style="3"/>
-    <col min="16" max="16" width="9.54285714285714" style="4" customWidth="1"/>
-    <col min="17" max="17" width="13" customWidth="1"/>
-    <col min="18" max="18" width="10" customWidth="1"/>
+    <col min="5" max="5" width="14.7142857142857" style="2" customWidth="1"/>
+    <col min="6" max="7" width="19.1809523809524" customWidth="1"/>
+    <col min="8" max="8" width="15.2666666666667" customWidth="1"/>
+    <col min="9" max="10" width="15.2666666666667" style="2" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="12.8190476190476" customWidth="1"/>
+    <col min="13" max="13" width="22.1809523809524" style="3" customWidth="1"/>
+    <col min="14" max="14" width="11.5428571428571" customWidth="1"/>
+    <col min="15" max="15" width="15.4571428571429" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="17" max="17" width="13.8190476190476" customWidth="1"/>
+    <col min="18" max="18" width="9.18095238095238" style="4"/>
+    <col min="19" max="19" width="9.54285714285714" style="5" customWidth="1"/>
+    <col min="20" max="20" width="13" customWidth="1"/>
+    <col min="21" max="21" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:22">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1298,7 +1291,7 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -1310,259 +1303,268 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="S1" s="5" t="s">
         <v>18</v>
       </c>
+      <c r="T1" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="9" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:22">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" s="2">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" s="3">
         <v>2</v>
-      </c>
-      <c r="K2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" t="s">
-        <v>26</v>
       </c>
       <c r="N2" t="s">
         <v>27</v>
       </c>
-      <c r="O2" s="3">
+      <c r="O2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>30</v>
+      </c>
+      <c r="R2" s="4">
         <v>1</v>
       </c>
-      <c r="P2" s="4">
+      <c r="S2" s="5">
         <v>480000</v>
       </c>
-      <c r="Q2">
+      <c r="T2">
         <v>480000</v>
       </c>
-      <c r="R2">
+      <c r="U2">
         <v>1</v>
       </c>
-      <c r="S2">
+      <c r="V2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:22">
       <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O3" s="3">
+        <v>22</v>
+      </c>
+      <c r="O3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>33</v>
+      </c>
+      <c r="R3" s="4">
         <v>2</v>
       </c>
-      <c r="P3" s="4">
+      <c r="S3" s="5">
         <v>1600</v>
       </c>
-      <c r="Q3">
+      <c r="T3">
         <v>2264000</v>
       </c>
-      <c r="R3">
+      <c r="U3">
         <v>1</v>
       </c>
-      <c r="S3">
+      <c r="V3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:22">
       <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="L4" t="s">
-        <v>31</v>
-      </c>
-      <c r="M4" t="s">
-        <v>32</v>
-      </c>
-      <c r="N4" t="s">
-        <v>33</v>
-      </c>
-      <c r="O4" s="3">
+        <v>22</v>
+      </c>
+      <c r="O4" t="s">
+        <v>34</v>
+      </c>
+      <c r="P4" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>36</v>
+      </c>
+      <c r="R4" s="4">
         <v>3</v>
       </c>
-      <c r="P4" s="4">
+      <c r="S4" s="5">
         <v>480000</v>
       </c>
-      <c r="Q4">
+      <c r="T4">
         <v>1797600</v>
       </c>
-      <c r="R4">
+      <c r="U4">
         <v>1</v>
       </c>
-      <c r="S4">
+      <c r="V4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:22">
       <c r="A5" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5" s="2">
+        <v>37</v>
+      </c>
+      <c r="M5" s="3">
         <v>2</v>
       </c>
-      <c r="K5" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" t="s">
-        <v>35</v>
-      </c>
-      <c r="M5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O5" s="3">
+      <c r="N5" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" t="s">
+        <v>38</v>
+      </c>
+      <c r="P5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R5" s="4">
         <v>3</v>
       </c>
-      <c r="P5" s="4">
+      <c r="S5" s="5">
         <v>230000</v>
       </c>
-      <c r="Q5">
-        <f>O5*P5</f>
+      <c r="T5">
+        <f>R5*S5</f>
         <v>690000</v>
       </c>
-      <c r="R5">
+      <c r="U5">
         <v>1</v>
       </c>
-      <c r="S5">
+      <c r="V5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:22">
       <c r="A6" t="s">
-        <v>37</v>
-      </c>
-      <c r="J6" s="2">
+        <v>40</v>
+      </c>
+      <c r="M6" s="3">
         <v>2</v>
       </c>
-      <c r="K6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6" t="s">
-        <v>38</v>
-      </c>
-      <c r="O6" s="3">
+      <c r="N6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" t="s">
+        <v>41</v>
+      </c>
+      <c r="R6" s="4">
         <v>1</v>
       </c>
-      <c r="P6" s="4">
+      <c r="S6" s="5">
         <v>200000</v>
       </c>
-      <c r="Q6">
-        <f t="shared" ref="Q6:Q8" si="0">O6*P6</f>
+      <c r="T6">
+        <f t="shared" ref="T6:T8" si="0">R6*S6</f>
         <v>200000</v>
       </c>
-      <c r="R6">
+      <c r="U6">
         <v>1</v>
       </c>
-      <c r="S6">
+      <c r="V6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:22">
       <c r="A7" t="s">
-        <v>37</v>
-      </c>
-      <c r="L7" t="s">
-        <v>39</v>
-      </c>
-      <c r="O7" s="3">
+        <v>40</v>
+      </c>
+      <c r="O7" t="s">
+        <v>42</v>
+      </c>
+      <c r="R7" s="4">
         <v>2</v>
       </c>
-      <c r="P7" s="4">
+      <c r="S7" s="5">
         <v>2900000</v>
       </c>
-      <c r="Q7">
+      <c r="T7">
         <f t="shared" si="0"/>
         <v>5800000</v>
       </c>
-      <c r="R7">
+      <c r="U7">
         <v>1</v>
       </c>
-      <c r="S7">
+      <c r="V7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:22">
       <c r="A8" t="s">
-        <v>37</v>
-      </c>
-      <c r="L8" t="s">
         <v>40</v>
       </c>
-      <c r="O8" s="3">
+      <c r="O8" t="s">
+        <v>43</v>
+      </c>
+      <c r="R8" s="4">
         <v>3</v>
       </c>
-      <c r="P8" s="4">
+      <c r="S8" s="5">
         <v>2300000</v>
       </c>
-      <c r="Q8">
+      <c r="T8">
         <f t="shared" si="0"/>
         <v>6900000</v>
       </c>
-      <c r="R8">
+      <c r="U8">
         <v>1</v>
       </c>
-      <c r="S8">
+      <c r="V8">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1585,47 +1587,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>